<commit_message>
Source contact email from ContactEmail sheet in SocialMedia.xlsx
Add a "ContactEmail" sheet (single Email column) and read it in
update-socialmedia.py, emitting window.CONTACT_EMAIL. index.html uses it
for the Web3Forms recipient (booking + contact forms) and the address
shown in the success message and terms, with a hardcoded fallback.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SocialMedia.xlsx
+++ b/SocialMedia.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SocialMedia" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ContactEmail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -491,4 +492,35 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>quicksoftwares.global@gmail.com</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>